<commit_message>
push customequipmentpackage & propertybreak & status
</commit_message>
<xml_diff>
--- a/ContinuationProject/Status.xlsx
+++ b/ContinuationProject/Status.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\DISCDEXPI\ContinuationProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88FADC31-FC4A-45A6-ADD1-51E7B60260F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9EFFD8C-F3BD-4122-9522-959E26BE5CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{975D681B-08B9-4F16-AF36-2B35AB80030D}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{975D681B-08B9-4F16-AF36-2B35AB80030D}"/>
   </bookViews>
   <sheets>
     <sheet name="Status" sheetId="4" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="86">
   <si>
     <t>DISC DEXPI Continuation Project - Status</t>
   </si>
@@ -260,9 +260,6 @@
     <t>03.11.2025</t>
   </si>
   <si>
-    <t>Issue fixed from old versions in-progress</t>
-  </si>
-  <si>
     <t>Keep as is with no new sub-types</t>
   </si>
   <si>
@@ -294,6 +291,22 @@
   </si>
   <si>
     <t>Available in DEXPI 2.0 xml. This is an issue for DEXPI group particularly for the overall conceptual model .. How shall OPCs be managed. (Signal &amp; Piping)</t>
+  </si>
+  <si>
+    <t>01.12.2025</t>
+  </si>
+  <si>
+    <t>To be delivered with Profile 3 due to NuclearSource</t>
+  </si>
+  <si>
+    <t>To be delivered with Profile 3 - need to change all other versions for reference info</t>
+  </si>
+  <si>
+    <t>Include example in Blueprint files - package only as new propertybreak model includes tie-ins.</t>
+  </si>
+  <si>
+    <t>Tonia to create ver 13 with custom equipment package &amp; joints. Tiein example not needed as this is covered by propertybreak.
+Update to existing propertybreak to cover model Profile 3</t>
   </si>
 </sst>
 </file>
@@ -303,7 +316,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;Done&quot;;&quot;&quot;;&quot;&quot;"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -362,6 +375,14 @@
       <color theme="3"/>
       <name val="Bookman Old Style"/>
       <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -423,7 +444,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" applyBorder="1" applyAlignment="1">
@@ -494,6 +515,7 @@
     <xf numFmtId="9" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Date" xfId="6" xr:uid="{2ABB41C5-3CC8-4E1C-85D9-965CF83E22BD}"/>
@@ -501,7 +523,7 @@
     <cellStyle name="Heading 1" xfId="3" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="4" builtinId="17"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Per cent" xfId="1" builtinId="5"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
     <cellStyle name="Title" xfId="2" builtinId="15"/>
   </cellStyles>
   <dxfs count="1">
@@ -850,34 +872,35 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{825F216F-6A2C-43F0-976D-4459909E096A}">
   <dimension ref="B1:BG49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="5.85546875" customWidth="1"/>
-    <col min="2" max="2" width="28.140625" customWidth="1"/>
-    <col min="3" max="3" width="56.7109375" customWidth="1"/>
-    <col min="4" max="4" width="29.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" style="20" customWidth="1"/>
-    <col min="6" max="6" width="14.42578125" customWidth="1"/>
-    <col min="7" max="7" width="19.7109375" customWidth="1"/>
+    <col min="1" max="1" width="5.86328125" customWidth="1"/>
+    <col min="2" max="2" width="28.1328125" customWidth="1"/>
+    <col min="3" max="3" width="56.73046875" customWidth="1"/>
+    <col min="4" max="4" width="29.73046875" customWidth="1"/>
+    <col min="5" max="5" width="14.59765625" style="20" customWidth="1"/>
+    <col min="6" max="6" width="14.3984375" customWidth="1"/>
+    <col min="7" max="7" width="19.73046875" customWidth="1"/>
     <col min="8" max="8" width="7" customWidth="1"/>
-    <col min="9" max="9" width="36.5703125" customWidth="1"/>
-    <col min="10" max="10" width="18.140625" style="22" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="16.85546875" style="22" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="36.59765625" customWidth="1"/>
+    <col min="10" max="10" width="18.1328125" style="22" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="16.86328125" style="22" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="15" style="22" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="19.85546875" style="22" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="17.7109375" style="22" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="19.86328125" style="22" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="17.73046875" style="22" hidden="1" customWidth="1"/>
     <col min="15" max="15" width="16" style="22" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="16.42578125" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="15.7109375" style="22" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="19.140625" style="22" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="15.42578125" style="22" customWidth="1"/>
-    <col min="20" max="20" width="20.28515625" style="22" customWidth="1"/>
-    <col min="21" max="21" width="13.85546875" style="22" customWidth="1"/>
-    <col min="22" max="22" width="15.5703125" style="22" customWidth="1"/>
-    <col min="23" max="36" width="9.140625" style="22"/>
+    <col min="16" max="16" width="16.3984375" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="15.73046875" style="22" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="19.1328125" style="22" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="15.3984375" style="22" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="20.265625" style="22" customWidth="1"/>
+    <col min="21" max="21" width="13.86328125" style="22" customWidth="1"/>
+    <col min="22" max="22" width="15.59765625" style="22" customWidth="1"/>
+    <col min="23" max="23" width="14.59765625" style="22" customWidth="1"/>
+    <col min="24" max="36" width="9.1328125" style="22"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:59" ht="35.25" x14ac:dyDescent="0.5">
+    <row r="1" spans="2:59" ht="34.9" x14ac:dyDescent="0.9">
       <c r="B1" s="16" t="s">
         <v>0</v>
       </c>
@@ -890,7 +913,7 @@
       <c r="I1" s="6"/>
       <c r="P1" s="26"/>
     </row>
-    <row r="2" spans="2:59" ht="9" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:59" ht="9" customHeight="1" x14ac:dyDescent="0.7">
       <c r="C2" s="6"/>
       <c r="D2" s="1"/>
       <c r="E2" s="17"/>
@@ -900,7 +923,7 @@
       <c r="I2" s="6"/>
       <c r="P2" s="26"/>
     </row>
-    <row r="3" spans="2:59" ht="19.5" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:59" ht="19.5" x14ac:dyDescent="0.6">
       <c r="B3" s="2" t="s">
         <v>19</v>
       </c>
@@ -956,15 +979,17 @@
         <v>69</v>
       </c>
       <c r="T3" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="U3" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="U3" s="27" t="s">
-        <v>75</v>
-      </c>
       <c r="V3" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="W3" s="20"/>
+        <v>78</v>
+      </c>
+      <c r="W3" s="30" t="s">
+        <v>81</v>
+      </c>
       <c r="X3" s="20"/>
       <c r="Y3" s="20"/>
       <c r="Z3" s="20"/>
@@ -1002,7 +1027,7 @@
       <c r="BF3" s="20"/>
       <c r="BG3" s="20"/>
     </row>
-    <row r="4" spans="2:59" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:59" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B4" s="9" t="s">
         <v>12</v>
       </c>
@@ -1017,17 +1042,17 @@
       </c>
       <c r="F4" s="9" t="str">
         <f>IF(G4=1,"Complete",IF(G4&lt;&gt;0,"In Progess","Not Started"))</f>
-        <v>In Progess</v>
+        <v>Complete</v>
       </c>
       <c r="G4" s="10">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="H4" s="11">
         <f>--(G4&gt;=1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J4" s="23">
         <v>0.3</v>
@@ -1068,8 +1093,11 @@
       <c r="V4" s="22">
         <v>0.98</v>
       </c>
-    </row>
-    <row r="5" spans="2:59" ht="30" x14ac:dyDescent="0.25">
+      <c r="W4" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:59" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B5" s="9" t="s">
         <v>12</v>
       </c>
@@ -1085,14 +1113,14 @@
         <v>In Progess</v>
       </c>
       <c r="G5" s="10">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="H5" s="11">
         <f t="shared" ref="H5:H49" si="1">--(G5&gt;=1)</f>
         <v>0</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J5" s="23">
         <v>0.75</v>
@@ -1133,8 +1161,11 @@
       <c r="V5" s="22">
         <v>0.98</v>
       </c>
-    </row>
-    <row r="6" spans="2:59" ht="30" x14ac:dyDescent="0.25">
+      <c r="W5" s="22">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="6" spans="2:59" x14ac:dyDescent="0.45">
       <c r="B6" s="9" t="s">
         <v>3</v>
       </c>
@@ -1196,8 +1227,11 @@
       <c r="V6" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="2:59" ht="30" x14ac:dyDescent="0.25">
+      <c r="W6" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:59" x14ac:dyDescent="0.45">
       <c r="B7" s="9" t="s">
         <v>3</v>
       </c>
@@ -1248,8 +1282,11 @@
       <c r="V7" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="2:59" x14ac:dyDescent="0.25">
+      <c r="W7" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:59" x14ac:dyDescent="0.45">
       <c r="B8" s="9" t="s">
         <v>3</v>
       </c>
@@ -1300,8 +1337,11 @@
       <c r="V8" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="2:59" ht="30" x14ac:dyDescent="0.25">
+      <c r="W8" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="2:59" x14ac:dyDescent="0.45">
       <c r="B9" s="9" t="s">
         <v>3</v>
       </c>
@@ -1324,7 +1364,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J9" s="23"/>
       <c r="P9" s="28"/>
@@ -1346,8 +1386,11 @@
       <c r="V9" s="22">
         <v>0.99</v>
       </c>
-    </row>
-    <row r="10" spans="2:59" x14ac:dyDescent="0.25">
+      <c r="W9" s="22">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="10" spans="2:59" x14ac:dyDescent="0.45">
       <c r="B10" s="9" t="s">
         <v>4</v>
       </c>
@@ -1406,8 +1449,11 @@
       <c r="V10" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="2:59" ht="45" x14ac:dyDescent="0.25">
+      <c r="W10" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="2:59" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B11" s="9" t="s">
         <v>5</v>
       </c>
@@ -1473,8 +1519,11 @@
       <c r="V11" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="2:59" x14ac:dyDescent="0.25">
+      <c r="W11" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="2:59" x14ac:dyDescent="0.45">
       <c r="B12" s="9" t="s">
         <v>5</v>
       </c>
@@ -1519,8 +1568,11 @@
       <c r="V12" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="2:59" ht="30" x14ac:dyDescent="0.25">
+      <c r="W12" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:59" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B13" s="9" t="s">
         <v>5</v>
       </c>
@@ -1536,14 +1588,14 @@
         <v>In Progess</v>
       </c>
       <c r="G13" s="10">
-        <v>0.95</v>
+        <v>0.98</v>
       </c>
       <c r="H13" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="J13" s="23"/>
       <c r="O13" s="22">
@@ -1570,8 +1622,11 @@
       <c r="V13" s="22">
         <v>0.95</v>
       </c>
-    </row>
-    <row r="14" spans="2:59" x14ac:dyDescent="0.25">
+      <c r="W13" s="22">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="14" spans="2:59" x14ac:dyDescent="0.45">
       <c r="B14" s="9" t="s">
         <v>6</v>
       </c>
@@ -1635,8 +1690,11 @@
       <c r="V14" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="2:59" ht="30" x14ac:dyDescent="0.25">
+      <c r="W14" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="2:59" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B15" s="9" t="s">
         <v>6</v>
       </c>
@@ -1659,7 +1717,7 @@
         <v>1</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J15" s="23">
         <v>0.7</v>
@@ -1700,8 +1758,11 @@
       <c r="V15" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="2:59" ht="75" x14ac:dyDescent="0.25">
+      <c r="W15" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:59" ht="57" x14ac:dyDescent="0.45">
       <c r="B16" s="9" t="s">
         <v>7</v>
       </c>
@@ -1724,7 +1785,7 @@
         <v>1</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J16" s="23">
         <v>0.2</v>
@@ -1765,8 +1826,11 @@
       <c r="V16" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="W16" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B17" s="9" t="s">
         <v>7</v>
       </c>
@@ -1808,8 +1872,11 @@
       <c r="V17" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W17" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B18" s="9" t="s">
         <v>7</v>
       </c>
@@ -1845,8 +1912,11 @@
       <c r="V18" s="22">
         <v>0.15</v>
       </c>
-    </row>
-    <row r="19" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W18" s="22">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="19" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B19" s="9" t="s">
         <v>7</v>
       </c>
@@ -1869,7 +1939,7 @@
         <v>1</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J19" s="23"/>
       <c r="P19" s="28"/>
@@ -1885,8 +1955,11 @@
       <c r="V19" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W19" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="2:23" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B20" s="9" t="s">
         <v>7</v>
       </c>
@@ -1902,11 +1975,14 @@
         <v>In Progess</v>
       </c>
       <c r="G20" s="10">
-        <v>0.2</v>
+        <v>0.98</v>
       </c>
       <c r="H20" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>83</v>
       </c>
       <c r="J20" s="23"/>
       <c r="P20" s="28"/>
@@ -1922,8 +1998,11 @@
       <c r="V20" s="22">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="21" spans="2:22" ht="105" x14ac:dyDescent="0.25">
+      <c r="W20" s="22">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="21" spans="2:23" ht="85.5" x14ac:dyDescent="0.45">
       <c r="B21" s="9" t="s">
         <v>8</v>
       </c>
@@ -1982,8 +2061,11 @@
       <c r="V21" s="22">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="22" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="W21" s="22">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="22" spans="2:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B22" s="9" t="s">
         <v>8</v>
       </c>
@@ -2039,8 +2121,11 @@
       <c r="V22" s="22">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="23" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W22" s="22">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="23" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B23" s="9" t="s">
         <v>8</v>
       </c>
@@ -2070,8 +2155,11 @@
       <c r="V23" s="22">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="24" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W23" s="22">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="24" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B24" s="9" t="s">
         <v>8</v>
       </c>
@@ -2094,12 +2182,12 @@
       <c r="J24" s="23"/>
       <c r="P24" s="28"/>
     </row>
-    <row r="25" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:23" ht="71.25" x14ac:dyDescent="0.45">
       <c r="B25" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="19">
@@ -2114,10 +2202,13 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="I25" s="6" t="s">
+        <v>85</v>
+      </c>
       <c r="J25" s="23"/>
       <c r="P25" s="28"/>
     </row>
-    <row r="26" spans="2:22" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:23" ht="49.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B26" s="9" t="s">
         <v>2</v>
       </c>
@@ -2181,8 +2272,11 @@
       <c r="V26" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W26" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B27" s="9" t="s">
         <v>2</v>
       </c>
@@ -2233,8 +2327,11 @@
       <c r="V27" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W27" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B28" s="9" t="s">
         <v>2</v>
       </c>
@@ -2279,8 +2376,11 @@
       <c r="V28" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W28" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B29" s="9" t="s">
         <v>2</v>
       </c>
@@ -2323,8 +2423,11 @@
       <c r="V29" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W29" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B30" s="9" t="s">
         <v>9</v>
       </c>
@@ -2347,7 +2450,7 @@
         <v>1</v>
       </c>
       <c r="I30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J30" s="23"/>
       <c r="L30" s="22">
@@ -2383,8 +2486,11 @@
       <c r="V30" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="W30" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="2:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B31" s="9" t="s">
         <v>9</v>
       </c>
@@ -2407,7 +2513,7 @@
         <v>1</v>
       </c>
       <c r="I31" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J31" s="23"/>
       <c r="L31" s="22">
@@ -2443,8 +2549,11 @@
       <c r="V31" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W31" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B32" s="9" t="s">
         <v>9</v>
       </c>
@@ -2484,8 +2593,11 @@
       <c r="V32" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W32" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B33" s="9" t="s">
         <v>9</v>
       </c>
@@ -2522,8 +2634,11 @@
       <c r="V33" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W33" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B34" s="9" t="s">
         <v>9</v>
       </c>
@@ -2560,8 +2675,11 @@
       <c r="V34" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W34" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B35" s="9" t="s">
         <v>36</v>
       </c>
@@ -2623,8 +2741,11 @@
       <c r="V35" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W35" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B36" s="9" t="s">
         <v>36</v>
       </c>
@@ -2675,8 +2796,11 @@
       <c r="V36" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W36" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B37" s="9" t="s">
         <v>36</v>
       </c>
@@ -2699,7 +2823,7 @@
         <v>0</v>
       </c>
       <c r="I37" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J37" s="23"/>
       <c r="O37" s="22">
@@ -2726,8 +2850,11 @@
       <c r="V37" s="22">
         <v>0.99</v>
       </c>
-    </row>
-    <row r="38" spans="2:22" ht="75" x14ac:dyDescent="0.25">
+      <c r="W37" s="22">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="38" spans="2:23" ht="57" x14ac:dyDescent="0.45">
       <c r="B38" s="9" t="s">
         <v>26</v>
       </c>
@@ -2791,8 +2918,11 @@
       <c r="V38" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="39" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W38" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B39" s="9" t="s">
         <v>26</v>
       </c>
@@ -2856,8 +2986,11 @@
       <c r="V39" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="40" spans="2:22" ht="30" x14ac:dyDescent="0.25">
+      <c r="W39" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="2:23" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B40" s="9" t="s">
         <v>26</v>
       </c>
@@ -2923,8 +3056,11 @@
       <c r="V40" s="22">
         <v>0.95</v>
       </c>
-    </row>
-    <row r="41" spans="2:22" ht="30" x14ac:dyDescent="0.25">
+      <c r="W40" s="22">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="41" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B41" s="9" t="s">
         <v>10</v>
       </c>
@@ -2986,8 +3122,11 @@
       <c r="V41" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="42" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W41" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B42" s="7" t="s">
         <v>28</v>
       </c>
@@ -3049,8 +3188,11 @@
       <c r="V42" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="43" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W42" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B43" s="7" t="s">
         <v>11</v>
       </c>
@@ -3112,8 +3254,11 @@
       <c r="V43" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W43" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B44" s="7" t="s">
         <v>15</v>
       </c>
@@ -3175,8 +3320,11 @@
       <c r="V44" s="22">
         <v>0.99</v>
       </c>
-    </row>
-    <row r="45" spans="2:22" ht="30" x14ac:dyDescent="0.25">
+      <c r="W44" s="22">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="45" spans="2:23" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B45" s="7" t="s">
         <v>15</v>
       </c>
@@ -3221,8 +3369,11 @@
       <c r="V45" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="46" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W45" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B46" s="7" t="s">
         <v>16</v>
       </c>
@@ -3284,8 +3435,11 @@
       <c r="V46" s="22">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="47" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W46" s="22">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="47" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B47" s="7" t="s">
         <v>17</v>
       </c>
@@ -3347,8 +3501,11 @@
       <c r="V47" s="22">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="48" spans="2:22" ht="45" x14ac:dyDescent="0.25">
+      <c r="W47" s="22">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="48" spans="2:23" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B48" t="s">
         <v>52</v>
       </c>
@@ -3402,8 +3559,11 @@
       <c r="V48" s="22">
         <v>1</v>
       </c>
-    </row>
-    <row r="49" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="W48" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="2:23" x14ac:dyDescent="0.45">
       <c r="B49" t="s">
         <v>54</v>
       </c>
@@ -3452,6 +3612,9 @@
         <v>1</v>
       </c>
       <c r="V49" s="22">
+        <v>1</v>
+      </c>
+      <c r="W49" s="22">
         <v>1</v>
       </c>
     </row>
@@ -3531,28 +3694,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23963325-1FFB-4B92-8120-662513F10342}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100C3422A7FFD03AF47B40E3148D61510DD" ma:contentTypeVersion="10" ma:contentTypeDescription="Opprett et nytt dokument." ma:contentTypeScope="" ma:versionID="93a5827b91256c075a5bcdb454d162de">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7ae1cb1b-b89b-4b35-8dc1-6b34b6393ff0" xmlns:ns3="b6192152-6ac4-477a-b62a-2f500fcdf3b6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="13127a08f307124b01356346b67d6a81" ns2:_="" ns3:_="">
     <xsd:import namespace="7ae1cb1b-b89b-4b35-8dc1-6b34b6393ff0"/>
@@ -3753,32 +3901,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CE334B8-DB7D-495D-B7B7-7E69CDC1BE08}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="7ae1cb1b-b89b-4b35-8dc1-6b34b6393ff0"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="b6192152-6ac4-477a-b62a-2f500fcdf3b6"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E81441C-10B0-478C-AED5-6210518ADFA7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4CED3C9C-630D-4C4B-A736-44AEC9EEC0A0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3795,4 +3933,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E81441C-10B0-478C-AED5-6210518ADFA7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CE334B8-DB7D-495D-B7B7-7E69CDC1BE08}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="7ae1cb1b-b89b-4b35-8dc1-6b34b6393ff0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="b6192152-6ac4-477a-b62a-2f500fcdf3b6"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update for blueprint 13, processVesselComponent and status
Need to update the other blueprints later.
</commit_message>
<xml_diff>
--- a/ContinuationProject/Status.xlsx
+++ b/ContinuationProject/Status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\DISCDEXPI\ContinuationProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9EFFD8C-F3BD-4122-9522-959E26BE5CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD5E4A89-837F-4A43-BAB3-2E69F020F183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{975D681B-08B9-4F16-AF36-2B35AB80030D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{975D681B-08B9-4F16-AF36-2B35AB80030D}"/>
   </bookViews>
   <sheets>
     <sheet name="Status" sheetId="4" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="88">
   <si>
     <t>DISC DEXPI Continuation Project - Status</t>
   </si>
@@ -307,6 +307,12 @@
   <si>
     <t>Tonia to create ver 13 with custom equipment package &amp; joints. Tiein example not needed as this is covered by propertybreak.
 Update to existing propertybreak to cover model Profile 3</t>
+  </si>
+  <si>
+    <t>Complete Workshop 12</t>
+  </si>
+  <si>
+    <t>12.12.2025</t>
   </si>
 </sst>
 </file>
@@ -871,36 +877,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{825F216F-6A2C-43F0-976D-4459909E096A}">
-  <dimension ref="B1:BG49"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="B1:BG50"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.86328125" customWidth="1"/>
-    <col min="2" max="2" width="28.1328125" customWidth="1"/>
-    <col min="3" max="3" width="56.73046875" customWidth="1"/>
-    <col min="4" max="4" width="29.73046875" customWidth="1"/>
-    <col min="5" max="5" width="14.59765625" style="20" customWidth="1"/>
-    <col min="6" max="6" width="14.3984375" customWidth="1"/>
-    <col min="7" max="7" width="19.73046875" customWidth="1"/>
+    <col min="1" max="1" width="5.85546875" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" customWidth="1"/>
+    <col min="3" max="3" width="56.7109375" customWidth="1"/>
+    <col min="4" max="4" width="29.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" style="20" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" customWidth="1"/>
+    <col min="7" max="7" width="19.7109375" customWidth="1"/>
     <col min="8" max="8" width="7" customWidth="1"/>
-    <col min="9" max="9" width="36.59765625" customWidth="1"/>
-    <col min="10" max="10" width="18.1328125" style="22" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="16.86328125" style="22" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="36.5703125" customWidth="1"/>
+    <col min="10" max="10" width="18.140625" style="22" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="16.85546875" style="22" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="15" style="22" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="19.86328125" style="22" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="17.73046875" style="22" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="19.85546875" style="22" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="17.7109375" style="22" hidden="1" customWidth="1"/>
     <col min="15" max="15" width="16" style="22" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="16.3984375" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="15.73046875" style="22" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="19.1328125" style="22" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="15.3984375" style="22" hidden="1" customWidth="1"/>
-    <col min="20" max="20" width="20.265625" style="22" customWidth="1"/>
-    <col min="21" max="21" width="13.86328125" style="22" customWidth="1"/>
-    <col min="22" max="22" width="15.59765625" style="22" customWidth="1"/>
-    <col min="23" max="23" width="14.59765625" style="22" customWidth="1"/>
-    <col min="24" max="36" width="9.1328125" style="22"/>
+    <col min="16" max="16" width="16.42578125" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="15.7109375" style="22" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="19.140625" style="22" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="15.42578125" style="22" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="20.28515625" style="22" customWidth="1"/>
+    <col min="21" max="21" width="13.85546875" style="22" customWidth="1"/>
+    <col min="22" max="22" width="15.5703125" style="22" customWidth="1"/>
+    <col min="23" max="23" width="14.5703125" style="22" customWidth="1"/>
+    <col min="24" max="24" width="16.85546875" style="22" customWidth="1"/>
+    <col min="25" max="36" width="9.140625" style="22"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:59" ht="34.9" x14ac:dyDescent="0.9">
+    <row r="1" spans="2:59" ht="35.25" x14ac:dyDescent="0.5">
       <c r="B1" s="16" t="s">
         <v>0</v>
       </c>
@@ -913,7 +920,7 @@
       <c r="I1" s="6"/>
       <c r="P1" s="26"/>
     </row>
-    <row r="2" spans="2:59" ht="9" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="2" spans="2:59" ht="9" customHeight="1" x14ac:dyDescent="0.4">
       <c r="C2" s="6"/>
       <c r="D2" s="1"/>
       <c r="E2" s="17"/>
@@ -923,7 +930,7 @@
       <c r="I2" s="6"/>
       <c r="P2" s="26"/>
     </row>
-    <row r="3" spans="2:59" ht="19.5" x14ac:dyDescent="0.6">
+    <row r="3" spans="2:59" ht="19.5" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
         <v>19</v>
       </c>
@@ -990,7 +997,9 @@
       <c r="W3" s="30" t="s">
         <v>81</v>
       </c>
-      <c r="X3" s="20"/>
+      <c r="X3" s="30" t="s">
+        <v>87</v>
+      </c>
       <c r="Y3" s="20"/>
       <c r="Z3" s="20"/>
       <c r="AA3" s="20"/>
@@ -1027,7 +1036,7 @@
       <c r="BF3" s="20"/>
       <c r="BG3" s="20"/>
     </row>
-    <row r="4" spans="2:59" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:59" ht="45" x14ac:dyDescent="0.25">
       <c r="B4" s="9" t="s">
         <v>12</v>
       </c>
@@ -1097,7 +1106,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:59" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:59" ht="30" x14ac:dyDescent="0.25">
       <c r="B5" s="9" t="s">
         <v>12</v>
       </c>
@@ -1165,7 +1174,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="6" spans="2:59" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:59" ht="30" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
         <v>3</v>
       </c>
@@ -1231,7 +1240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:59" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:59" ht="30" x14ac:dyDescent="0.25">
       <c r="B7" s="9" t="s">
         <v>3</v>
       </c>
@@ -1286,7 +1295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:59" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:59" ht="30" x14ac:dyDescent="0.25">
       <c r="B8" s="9" t="s">
         <v>3</v>
       </c>
@@ -1341,7 +1350,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:59" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:59" ht="30" x14ac:dyDescent="0.25">
       <c r="B9" s="9" t="s">
         <v>3</v>
       </c>
@@ -1390,7 +1399,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="10" spans="2:59" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B10" s="9" t="s">
         <v>4</v>
       </c>
@@ -1453,7 +1462,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:59" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:59" ht="45" x14ac:dyDescent="0.25">
       <c r="B11" s="9" t="s">
         <v>5</v>
       </c>
@@ -1523,7 +1532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:59" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B12" s="9" t="s">
         <v>5</v>
       </c>
@@ -1572,7 +1581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:59" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:59" ht="30" x14ac:dyDescent="0.25">
       <c r="B13" s="9" t="s">
         <v>5</v>
       </c>
@@ -1626,7 +1635,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="14" spans="2:59" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:59" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
         <v>6</v>
       </c>
@@ -1694,7 +1703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:59" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:59" ht="30" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
         <v>6</v>
       </c>
@@ -1762,7 +1771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:59" ht="57" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:59" ht="75" x14ac:dyDescent="0.25">
       <c r="B16" s="9" t="s">
         <v>7</v>
       </c>
@@ -1830,7 +1839,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="9" t="s">
         <v>7</v>
       </c>
@@ -1876,7 +1885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B18" s="9" t="s">
         <v>7</v>
       </c>
@@ -1916,7 +1925,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="19" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B19" s="9" t="s">
         <v>7</v>
       </c>
@@ -1959,7 +1968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:23" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:23" ht="45" x14ac:dyDescent="0.25">
       <c r="B20" s="9" t="s">
         <v>7</v>
       </c>
@@ -2002,7 +2011,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="21" spans="2:23" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:23" ht="90" x14ac:dyDescent="0.25">
       <c r="B21" s="9" t="s">
         <v>8</v>
       </c>
@@ -2015,14 +2024,14 @@
       </c>
       <c r="F21" s="9" t="str">
         <f t="shared" si="0"/>
-        <v>In Progess</v>
+        <v>Complete</v>
       </c>
       <c r="G21" s="10">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="H21" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" s="6" t="s">
         <v>51</v>
@@ -2065,7 +2074,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="22" spans="2:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="9" t="s">
         <v>8</v>
       </c>
@@ -2078,14 +2087,14 @@
       </c>
       <c r="F22" s="9" t="str">
         <f t="shared" si="0"/>
-        <v>In Progess</v>
+        <v>Complete</v>
       </c>
       <c r="G22" s="10">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="H22" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" s="23"/>
       <c r="L22" s="22">
@@ -2125,7 +2134,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="23" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B23" s="9" t="s">
         <v>8</v>
       </c>
@@ -2159,7 +2168,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="24" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B24" s="9" t="s">
         <v>8</v>
       </c>
@@ -2182,7 +2191,7 @@
       <c r="J24" s="23"/>
       <c r="P24" s="28"/>
     </row>
-    <row r="25" spans="2:23" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:23" ht="90" x14ac:dyDescent="0.25">
       <c r="B25" s="9" t="s">
         <v>8</v>
       </c>
@@ -2195,9 +2204,11 @@
       </c>
       <c r="F25" s="9" t="str">
         <f t="shared" si="0"/>
-        <v>Not Started</v>
-      </c>
-      <c r="G25" s="10"/>
+        <v>In Progess</v>
+      </c>
+      <c r="G25" s="10">
+        <v>0.15</v>
+      </c>
       <c r="H25" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2208,7 +2219,7 @@
       <c r="J25" s="23"/>
       <c r="P25" s="28"/>
     </row>
-    <row r="26" spans="2:23" ht="49.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:23" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="9" t="s">
         <v>2</v>
       </c>
@@ -2276,7 +2287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B27" s="9" t="s">
         <v>2</v>
       </c>
@@ -2331,7 +2342,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B28" s="9" t="s">
         <v>2</v>
       </c>
@@ -2380,7 +2391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B29" s="9" t="s">
         <v>2</v>
       </c>
@@ -2427,7 +2438,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B30" s="9" t="s">
         <v>9</v>
       </c>
@@ -2490,7 +2501,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="2:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="9" t="s">
         <v>9</v>
       </c>
@@ -2553,7 +2564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B32" s="9" t="s">
         <v>9</v>
       </c>
@@ -2597,7 +2608,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B33" s="9" t="s">
         <v>9</v>
       </c>
@@ -2638,7 +2649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B34" s="9" t="s">
         <v>9</v>
       </c>
@@ -2679,7 +2690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B35" s="9" t="s">
         <v>36</v>
       </c>
@@ -2745,7 +2756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B36" s="9" t="s">
         <v>36</v>
       </c>
@@ -2800,7 +2811,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="37" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B37" s="9" t="s">
         <v>36</v>
       </c>
@@ -2854,7 +2865,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="38" spans="2:23" ht="57" x14ac:dyDescent="0.45">
+    <row r="38" spans="2:23" ht="75" x14ac:dyDescent="0.25">
       <c r="B38" s="9" t="s">
         <v>26</v>
       </c>
@@ -2922,7 +2933,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="39" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B39" s="9" t="s">
         <v>26</v>
       </c>
@@ -2990,7 +3001,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="2:23" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="40" spans="2:23" ht="30" x14ac:dyDescent="0.25">
       <c r="B40" s="9" t="s">
         <v>26</v>
       </c>
@@ -3060,7 +3071,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="41" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="41" spans="2:23" ht="30" x14ac:dyDescent="0.25">
       <c r="B41" s="9" t="s">
         <v>10</v>
       </c>
@@ -3126,7 +3137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="42" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B42" s="7" t="s">
         <v>28</v>
       </c>
@@ -3192,7 +3203,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="43" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B43" s="7" t="s">
         <v>11</v>
       </c>
@@ -3258,7 +3269,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="44" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B44" s="7" t="s">
         <v>15</v>
       </c>
@@ -3324,7 +3335,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="45" spans="2:23" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="45" spans="2:23" ht="30" x14ac:dyDescent="0.25">
       <c r="B45" s="7" t="s">
         <v>15</v>
       </c>
@@ -3373,7 +3384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="46" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B46" s="7" t="s">
         <v>16</v>
       </c>
@@ -3439,7 +3450,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="47" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="47" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B47" s="7" t="s">
         <v>17</v>
       </c>
@@ -3455,7 +3466,7 @@
         <v>In Progess</v>
       </c>
       <c r="G47" s="13">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="H47" s="11">
         <f t="shared" si="1"/>
@@ -3505,7 +3516,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="48" spans="2:23" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="48" spans="2:23" ht="45" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
         <v>52</v>
       </c>
@@ -3563,7 +3574,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="2:23" x14ac:dyDescent="0.45">
+    <row r="49" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
         <v>54</v>
       </c>
@@ -3618,9 +3629,52 @@
         <v>1</v>
       </c>
     </row>
+    <row r="50" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>86</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E50" s="20">
+        <v>45980</v>
+      </c>
+      <c r="F50" s="9" t="str">
+        <f t="shared" ref="F50" si="4">IF(G50=1,"Complete",IF(G50&lt;&gt;0,"In Progess","Not Started"))</f>
+        <v>Complete</v>
+      </c>
+      <c r="G50" s="24">
+        <v>1</v>
+      </c>
+      <c r="H50" s="25">
+        <f t="shared" ref="H50" si="5">--(G50&gt;=1)</f>
+        <v>1</v>
+      </c>
+      <c r="M50" s="22">
+        <v>1</v>
+      </c>
+      <c r="N50" s="22">
+        <v>1</v>
+      </c>
+      <c r="O50" s="22">
+        <v>1</v>
+      </c>
+      <c r="P50" s="24">
+        <v>1</v>
+      </c>
+      <c r="Q50" s="22">
+        <v>1</v>
+      </c>
+      <c r="R50" s="22">
+        <v>1</v>
+      </c>
+      <c r="S50" s="22">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="B3:BG47" xr:uid="{825F216F-6A2C-43F0-976D-4459909E096A}"/>
-  <conditionalFormatting sqref="G4:G49">
+  <conditionalFormatting sqref="G4:G50">
     <cfRule type="dataBar" priority="2">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -3642,7 +3696,7 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Start Date in this column under this heading" sqref="J3" xr:uid="{B097AD3D-83FE-4DB6-8AA6-82D58880DEE8}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Icon indicator for task completion in this column under this heading is automatically updated as tasks complete" sqref="H3" xr:uid="{E57FD015-A334-4A3D-9540-92E1D8A918A9}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Task in this column under this heading. Use heading filters to find specific entries" sqref="B3:D3" xr:uid="{6FDCA3F5-F6F1-45FB-8AE7-E90C5E60E365}"/>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Select entry from the list. Select CANCEL, then press ALT+DOWN ARROW to navigate the list. Select ENTER to make selection" sqref="F4:F49" xr:uid="{90892BC2-20A5-4151-9864-7558336C2FE7}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Select entry from the list. Select CANCEL, then press ALT+DOWN ARROW to navigate the list. Select ENTER to make selection" sqref="F4:F50" xr:uid="{90892BC2-20A5-4151-9864-7558336C2FE7}">
       <formula1>"Not Started, In Progress, Deferred, Complete"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3664,7 +3718,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>G4:G49</xm:sqref>
+          <xm:sqref>G4:G50</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="iconSet" priority="22" id="{E713B901-0E7B-40B8-A534-1C73C66CF397}">
@@ -3683,7 +3737,7 @@
               <x14:cfIcon iconSet="3Symbols" iconId="2"/>
             </x14:iconSet>
           </x14:cfRule>
-          <xm:sqref>H4:H49</xm:sqref>
+          <xm:sqref>H4:H50</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -3694,7 +3748,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23963325-1FFB-4B92-8120-662513F10342}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3902,18 +3956,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3936,14 +3990,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E81441C-10B0-478C-AED5-6210518ADFA7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CE334B8-DB7D-495D-B7B7-7E69CDC1BE08}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -3958,4 +4004,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E81441C-10B0-478C-AED5-6210518ADFA7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>